<commit_message>
MANTIS hardware design completed and first sample PCB ordered
</commit_message>
<xml_diff>
--- a/01_HARDWARE_ALTIUM/Project Outputs for ZASS_MANTIS/BOM/Bill of Materials-ZASS_MANTIS.xlsx
+++ b/01_HARDWARE_ALTIUM/Project Outputs for ZASS_MANTIS/BOM/Bill of Materials-ZASS_MANTIS.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29628"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ALPER\Desktop\REPO\ELS_CONTROL\01_HARDWARE_ALTIUM\Project Outputs for ZASS_MANTIS\BOM\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{E70EA66C-CC2A-4FCB-BCE4-759291DBCCAB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{A477ED74-EF0E-4242-A2CC-AC4576794F69}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{523E9F48-BC3E-4E04-BE55-19B2D58BE725}"/>
+    <workbookView xWindow="3510" yWindow="3510" windowWidth="21600" windowHeight="11295" xr2:uid="{89992401-646C-4472-9375-03254CDD27AF}"/>
   </bookViews>
   <sheets>
     <sheet name="Bill of Materials-ZASS_MANTIS" sheetId="1" r:id="rId1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="151" uniqueCount="135">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="161" uniqueCount="145">
   <si>
     <t>Comment</t>
   </si>
@@ -107,7 +107,7 @@
     <t>CAP CER X7R 0805</t>
   </si>
   <si>
-    <t>C8, C9, C10, C11, C12, C14, C15</t>
+    <t>C8, C9, C11, C12, C14, C15</t>
   </si>
   <si>
     <t>FP-CC0805-EA-MFG</t>
@@ -131,19 +131,43 @@
     <t>CMP-22017-000030-1</t>
   </si>
   <si>
-    <t>SZNUP2105LT3G</t>
-  </si>
-  <si>
-    <t>Dual Line CAN Bus Protector, 3-Pin SOT-23, Pb-Free, Tape and Reel</t>
-  </si>
-  <si>
-    <t>D2, D3</t>
-  </si>
-  <si>
-    <t>ONSC-SOT-23-3-318-08_V</t>
-  </si>
-  <si>
-    <t>CMP-1063-00169-1</t>
+    <t>ESDCAN06-2BWY</t>
+  </si>
+  <si>
+    <t>TVS Diode (Bi-directional)</t>
+  </si>
+  <si>
+    <t>D2, D4</t>
+  </si>
+  <si>
+    <t>SOT65P210X110-3N</t>
+  </si>
+  <si>
+    <t>SM712.TCT</t>
+  </si>
+  <si>
+    <t>Asymmetrical TVS Diode for Extended Common-Mode RS-485, 400 W, -55 to 125 degC, 3-Pin SOT23, RoHS, Tape and Reel</t>
+  </si>
+  <si>
+    <t>D3</t>
+  </si>
+  <si>
+    <t>SMTC-SOT23-3_V</t>
+  </si>
+  <si>
+    <t>CMP-2000-05357-1</t>
+  </si>
+  <si>
+    <t>1N4007WS</t>
+  </si>
+  <si>
+    <t>Diode</t>
+  </si>
+  <si>
+    <t>D5</t>
+  </si>
+  <si>
+    <t>SOD2613X110N</t>
   </si>
   <si>
     <t>STM32G0B1CBT6TR</t>
@@ -173,22 +197,13 @@
     <t>IC3</t>
   </si>
   <si>
-    <t>74HC4053FT</t>
-  </si>
-  <si>
-    <t>IC4</t>
-  </si>
-  <si>
-    <t>SOP65P640X120-16N</t>
-  </si>
-  <si>
     <t>B2B-XH-A(LF)(SN)</t>
   </si>
   <si>
     <t>CONN HEADER VERT 2POS 2.5MM</t>
   </si>
   <si>
-    <t>J1, J3</t>
+    <t>J1, J3, J9</t>
   </si>
   <si>
     <t>FP-B2B-XH-A_LF_SN-MFG</t>
@@ -212,10 +227,25 @@
     <t>CMP-17439-000304-1</t>
   </si>
   <si>
+    <t>B3B-XH-A(LF)(SN)</t>
+  </si>
+  <si>
+    <t>CONN HEADER VERT 3POS 2.5MM</t>
+  </si>
+  <si>
+    <t>J4, J8</t>
+  </si>
+  <si>
+    <t>FP-B3B-XH-A_LF_SN-MFG</t>
+  </si>
+  <si>
+    <t>CMP-17439-000014-3</t>
+  </si>
+  <si>
     <t>S2B-XH-A(LF)(SN)</t>
   </si>
   <si>
-    <t>J4, J5</t>
+    <t>J5</t>
   </si>
   <si>
     <t>B6B-XH-AM(LF)(SN)</t>
@@ -308,7 +338,7 @@
     <t>CRGCQ0603 120Ω 1% ±100ppm/°C 75V</t>
   </si>
   <si>
-    <t>R2</t>
+    <t>R2, R27, R28</t>
   </si>
   <si>
     <t>CMP-03211-001601-1</t>
@@ -320,7 +350,7 @@
     <t>RES Thick Film, 4.7kΩ, 1%, 0.1W, 100ppm/°C, 0603</t>
   </si>
   <si>
-    <t>R6, R7, R8, R9</t>
+    <t>R6, R7, R8, R9, R14</t>
   </si>
   <si>
     <t>FP-CRCW0603-e3-IPC_A</t>
@@ -329,46 +359,46 @@
     <t>CMP-1666-00019-3</t>
   </si>
   <si>
+    <t>CRGCQ1206F1K0</t>
+  </si>
+  <si>
+    <t>CRGCQ1206 1KΩ 0.25W 1% ±100ppm/°C 200V</t>
+  </si>
+  <si>
+    <t>R10</t>
+  </si>
+  <si>
+    <t>FP-CRGCQ1206-IPC_C</t>
+  </si>
+  <si>
+    <t>CMP-03211-006592-1</t>
+  </si>
+  <si>
+    <t>CRGCQ0603F1K2</t>
+  </si>
+  <si>
+    <t>CRGCQ 0603 1K2 1%</t>
+  </si>
+  <si>
+    <t>R16, R17, R19</t>
+  </si>
+  <si>
+    <t>CMP-03211-000516-1</t>
+  </si>
+  <si>
     <t>RC3216J202CS</t>
   </si>
   <si>
     <t>Res Thick Film 1206 2kΩ 5% 0.25W ±100ppm/°C Molded SMD T/R</t>
   </si>
   <si>
-    <t>R10, R18</t>
+    <t>R18</t>
   </si>
   <si>
     <t>FP-RC3216-IPC_A</t>
   </si>
   <si>
     <t>CMP-13261-004107-1</t>
-  </si>
-  <si>
-    <t>CRGP0805F33R</t>
-  </si>
-  <si>
-    <t>CRGP0805 33Ω 0.33W ±100ppm/°C 1% 150V</t>
-  </si>
-  <si>
-    <t>R14</t>
-  </si>
-  <si>
-    <t>FP-CRGP0805-IPC_C</t>
-  </si>
-  <si>
-    <t>CMP-03211-005140-1</t>
-  </si>
-  <si>
-    <t>CRGCQ0603F1K2</t>
-  </si>
-  <si>
-    <t>CRGCQ 0603 1K2 1%</t>
-  </si>
-  <si>
-    <t>R16, R17, R19</t>
-  </si>
-  <si>
-    <t>CMP-03211-000516-1</t>
   </si>
   <si>
     <t>PTS647SK38SMTR2LFS</t>
@@ -839,8 +869,8 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BCBB0A43-1D72-4F96-B0E7-23C988A198FD}">
-  <dimension ref="A1:F30"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7AC64F12-FF51-4495-98B2-DC5136FB484C}">
+  <dimension ref="A1:F32"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="6" width="19.7109375" customWidth="1"/>
@@ -943,7 +973,7 @@
         <v>24</v>
       </c>
       <c r="F5" s="1">
-        <v>7</v>
+        <v>6</v>
       </c>
     </row>
     <row r="6" spans="1:6" x14ac:dyDescent="0.25">
@@ -980,7 +1010,7 @@
         <v>33</v>
       </c>
       <c r="E7" s="2" t="s">
-        <v>34</v>
+        <v>30</v>
       </c>
       <c r="F7" s="1">
         <v>2</v>
@@ -988,19 +1018,19 @@
     </row>
     <row r="8" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A8" s="2" t="s">
+        <v>34</v>
+      </c>
+      <c r="B8" s="2" t="s">
         <v>35</v>
       </c>
-      <c r="B8" s="2" t="s">
+      <c r="C8" s="2" t="s">
         <v>36</v>
       </c>
-      <c r="C8" s="2" t="s">
+      <c r="D8" s="2" t="s">
         <v>37</v>
       </c>
-      <c r="D8" s="2" t="s">
+      <c r="E8" s="2" t="s">
         <v>38</v>
-      </c>
-      <c r="E8" s="2" t="s">
-        <v>35</v>
       </c>
       <c r="F8" s="1">
         <v>1</v>
@@ -1011,36 +1041,36 @@
         <v>39</v>
       </c>
       <c r="B9" s="2" t="s">
-        <v>36</v>
+        <v>40</v>
       </c>
       <c r="C9" s="2" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="D9" s="2" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="E9" s="2" t="s">
         <v>39</v>
       </c>
       <c r="F9" s="1">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="10" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A10" s="2" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="B10" s="2" t="s">
-        <v>36</v>
+        <v>44</v>
       </c>
       <c r="C10" s="2" t="s">
+        <v>45</v>
+      </c>
+      <c r="D10" s="2" t="s">
+        <v>46</v>
+      </c>
+      <c r="E10" s="2" t="s">
         <v>43</v>
-      </c>
-      <c r="D10" s="2" t="s">
-        <v>41</v>
-      </c>
-      <c r="E10" s="2" t="s">
-        <v>42</v>
       </c>
       <c r="F10" s="1">
         <v>1</v>
@@ -1048,42 +1078,42 @@
     </row>
     <row r="11" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A11" s="2" t="s">
+        <v>47</v>
+      </c>
+      <c r="B11" s="2" t="s">
         <v>44</v>
       </c>
-      <c r="B11" s="2" t="s">
-        <v>36</v>
-      </c>
       <c r="C11" s="2" t="s">
-        <v>45</v>
+        <v>48</v>
       </c>
       <c r="D11" s="2" t="s">
-        <v>46</v>
+        <v>49</v>
       </c>
       <c r="E11" s="2" t="s">
-        <v>44</v>
+        <v>47</v>
       </c>
       <c r="F11" s="1">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="12" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A12" s="2" t="s">
-        <v>47</v>
+        <v>50</v>
       </c>
       <c r="B12" s="2" t="s">
-        <v>48</v>
+        <v>44</v>
       </c>
       <c r="C12" s="2" t="s">
+        <v>51</v>
+      </c>
+      <c r="D12" s="2" t="s">
         <v>49</v>
       </c>
-      <c r="D12" s="2" t="s">
+      <c r="E12" s="2" t="s">
         <v>50</v>
       </c>
-      <c r="E12" s="2" t="s">
-        <v>51</v>
-      </c>
       <c r="F12" s="1">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="13" spans="1:6" x14ac:dyDescent="0.25">
@@ -1103,7 +1133,7 @@
         <v>56</v>
       </c>
       <c r="F13" s="1">
-        <v>1</v>
+        <v>3</v>
       </c>
     </row>
     <row r="14" spans="1:6" x14ac:dyDescent="0.25">
@@ -1111,56 +1141,56 @@
         <v>57</v>
       </c>
       <c r="B14" s="2" t="s">
-        <v>48</v>
+        <v>58</v>
       </c>
       <c r="C14" s="2" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="D14" s="2" t="s">
-        <v>50</v>
+        <v>60</v>
       </c>
       <c r="E14" s="2" t="s">
-        <v>51</v>
+        <v>61</v>
       </c>
       <c r="F14" s="1">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="15" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A15" s="2" t="s">
-        <v>59</v>
+        <v>62</v>
       </c>
       <c r="B15" s="2" t="s">
-        <v>60</v>
+        <v>63</v>
       </c>
       <c r="C15" s="2" t="s">
-        <v>61</v>
+        <v>64</v>
       </c>
       <c r="D15" s="2" t="s">
-        <v>62</v>
+        <v>65</v>
       </c>
       <c r="E15" s="2" t="s">
-        <v>63</v>
+        <v>66</v>
       </c>
       <c r="F15" s="1">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="16" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A16" s="2" t="s">
-        <v>64</v>
+        <v>67</v>
       </c>
       <c r="B16" s="2" t="s">
-        <v>65</v>
+        <v>53</v>
       </c>
       <c r="C16" s="2" t="s">
-        <v>66</v>
+        <v>68</v>
       </c>
       <c r="D16" s="2" t="s">
-        <v>67</v>
+        <v>55</v>
       </c>
       <c r="E16" s="2" t="s">
-        <v>64</v>
+        <v>56</v>
       </c>
       <c r="F16" s="1">
         <v>1</v>
@@ -1168,19 +1198,19 @@
     </row>
     <row r="17" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A17" s="2" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="B17" s="2" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="C17" s="2" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="D17" s="2" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="E17" s="2" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="F17" s="1">
         <v>1</v>
@@ -1188,19 +1218,19 @@
     </row>
     <row r="18" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A18" s="2" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="B18" s="2" t="s">
+        <v>75</v>
+      </c>
+      <c r="C18" s="2" t="s">
+        <v>76</v>
+      </c>
+      <c r="D18" s="2" t="s">
+        <v>77</v>
+      </c>
+      <c r="E18" s="2" t="s">
         <v>74</v>
-      </c>
-      <c r="C18" s="2" t="s">
-        <v>75</v>
-      </c>
-      <c r="D18" s="2" t="s">
-        <v>76</v>
-      </c>
-      <c r="E18" s="2" t="s">
-        <v>73</v>
       </c>
       <c r="F18" s="1">
         <v>1</v>
@@ -1208,19 +1238,19 @@
     </row>
     <row r="19" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A19" s="2" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="B19" s="2" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="C19" s="2" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="D19" s="2" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="E19" s="2" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="F19" s="1">
         <v>1</v>
@@ -1228,22 +1258,22 @@
     </row>
     <row r="20" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A20" s="2" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="B20" s="2" t="s">
+        <v>84</v>
+      </c>
+      <c r="C20" s="2" t="s">
+        <v>85</v>
+      </c>
+      <c r="D20" s="2" t="s">
+        <v>86</v>
+      </c>
+      <c r="E20" s="2" t="s">
         <v>83</v>
       </c>
-      <c r="C20" s="2" t="s">
-        <v>84</v>
-      </c>
-      <c r="D20" s="2" t="s">
-        <v>85</v>
-      </c>
-      <c r="E20" s="2" t="s">
-        <v>86</v>
-      </c>
       <c r="F20" s="1">
-        <v>8</v>
+        <v>1</v>
       </c>
     </row>
     <row r="21" spans="1:6" x14ac:dyDescent="0.25">
@@ -1257,10 +1287,10 @@
         <v>89</v>
       </c>
       <c r="D21" s="2" t="s">
-        <v>85</v>
+        <v>90</v>
       </c>
       <c r="E21" s="2" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="F21" s="1">
         <v>1</v>
@@ -1268,42 +1298,42 @@
     </row>
     <row r="22" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A22" s="2" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="B22" s="2" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="C22" s="2" t="s">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="D22" s="2" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="E22" s="2" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="F22" s="1">
-        <v>4</v>
+        <v>8</v>
       </c>
     </row>
     <row r="23" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A23" s="2" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="B23" s="2" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="C23" s="2" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="D23" s="2" t="s">
-        <v>99</v>
+        <v>95</v>
       </c>
       <c r="E23" s="2" t="s">
         <v>100</v>
       </c>
       <c r="F23" s="1">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="24" spans="1:6" x14ac:dyDescent="0.25">
@@ -1323,7 +1353,7 @@
         <v>105</v>
       </c>
       <c r="F24" s="1">
-        <v>1</v>
+        <v>5</v>
       </c>
     </row>
     <row r="25" spans="1:6" x14ac:dyDescent="0.25">
@@ -1337,33 +1367,33 @@
         <v>108</v>
       </c>
       <c r="D25" s="2" t="s">
-        <v>85</v>
+        <v>109</v>
       </c>
       <c r="E25" s="2" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="F25" s="1">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="26" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A26" s="2" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="B26" s="2" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="C26" s="2" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="D26" s="2" t="s">
-        <v>113</v>
+        <v>95</v>
       </c>
       <c r="E26" s="2" t="s">
         <v>114</v>
       </c>
       <c r="F26" s="1">
-        <v>1</v>
+        <v>3</v>
       </c>
     </row>
     <row r="27" spans="1:6" x14ac:dyDescent="0.25">
@@ -1443,6 +1473,46 @@
         <v>134</v>
       </c>
       <c r="F30" s="1">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="31" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A31" s="2" t="s">
+        <v>135</v>
+      </c>
+      <c r="B31" s="2" t="s">
+        <v>136</v>
+      </c>
+      <c r="C31" s="2" t="s">
+        <v>137</v>
+      </c>
+      <c r="D31" s="2" t="s">
+        <v>138</v>
+      </c>
+      <c r="E31" s="2" t="s">
+        <v>139</v>
+      </c>
+      <c r="F31" s="1">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="32" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A32" s="2" t="s">
+        <v>140</v>
+      </c>
+      <c r="B32" s="2" t="s">
+        <v>141</v>
+      </c>
+      <c r="C32" s="2" t="s">
+        <v>142</v>
+      </c>
+      <c r="D32" s="2" t="s">
+        <v>143</v>
+      </c>
+      <c r="E32" s="2" t="s">
+        <v>144</v>
+      </c>
+      <c r="F32" s="1">
         <v>1</v>
       </c>
     </row>

</xml_diff>